<commit_message>
testing order page & adding requirements
</commit_message>
<xml_diff>
--- a/Bug_Report.xlsx
+++ b/Bug_Report.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="57">
   <si>
     <t xml:space="preserve">Bug ID</t>
   </si>
@@ -74,7 +74,7 @@
   </si>
   <si>
     <t xml:space="preserve">1. Open the home page.
-2. In the name input field, type only spaces (e.g. "    ").
+2. In the name input field, type only spaces.
 3. Check if the "Start ordering" button appears.
 4. Click the "Start ordering" button.
 </t>
@@ -126,7 +126,7 @@
     <t xml:space="preserve">Hero pizza image element exists, but the browser shows a broken-image icon.</t>
   </si>
   <si>
-    <t xml:space="preserve">In progress</t>
+    <t xml:space="preserve">Resolved</t>
   </si>
   <si>
     <t xml:space="preserve">Test Team</t>
@@ -138,17 +138,96 @@
     <t xml:space="preserve">22-Nov-2025</t>
   </si>
   <si>
-    <t xml:space="preserve">Image URL appears to be invalid or expired. </t>
+    <t xml:space="preserve">Fixed by updating the hero image URL to a valid resource.
+Re-tested: image displays correctly and automated test passed.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BUG-003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Customer name field on order page is editable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">On the order page, the customer Name field is editable. 
+The user can change the name that was originally entered on the home page, 
+which violates the requirement that the customer name must remain fixed once chosen.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. On the home page, enter a valid name and click "Start ordering".
+2. Add a pizza to the cart, go to the cart, then click "Order pizzas" to open the order page.
+3. Inspect the Name field on the order page.
+4. Attempt to click inside the Name field and modify its value.
+5. Try to type a different name or clear the field.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Name field is read-only or disabled.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Name field is editable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adhm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Front-end Team</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Name input on the order page is implemented as a normal editable text field.
+Likely missing 'readonly' or 'disabled' attribute, or missing logic to prevent editing.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Requirement breach: name should be fixed after being entered on the home page.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BUG-004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Get position" button on order page does not fill address field</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The "Get position" feature on the order page fails to populate the address field.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Navigate to the order page.
+2. Ensure the Address field is empty.
+3. Click on the "Get position" button.
+4. Wait for the result of the location/address retrieval.
+5. Check the Address field value.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">After clicking "Get position", the application retrieves the user position successfully.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">After clicking "Get position", the Address field remains empty.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Major</t>
+  </si>
+  <si>
+    <t xml:space="preserve">High</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saif</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Likely failure in geolocation or in fetching the API</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="General"/>
+    <numFmt numFmtId="165" formatCode="mm/dd/yy"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -199,15 +278,43 @@
     </font>
     <font>
       <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="0"/>
       <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Ubuntu"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="0"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="0"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="6">
@@ -290,7 +397,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="33">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -347,7 +454,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -359,31 +466,67 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -700,7 +843,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="120.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="121.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
         <v>14</v>
       </c>
@@ -758,7 +901,7 @@
       <c r="M3" s="11"/>
       <c r="N3" s="12"/>
     </row>
-    <row r="4" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="106.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
         <v>26</v>
       </c>
@@ -816,69 +959,123 @@
       <c r="M5" s="11"/>
       <c r="N5" s="12"/>
     </row>
-    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="17"/>
-      <c r="B6" s="17"/>
-      <c r="C6" s="17"/>
-      <c r="D6" s="17"/>
-      <c r="E6" s="17"/>
-      <c r="F6" s="17"/>
-      <c r="G6" s="17"/>
-      <c r="H6" s="17"/>
-      <c r="I6" s="17"/>
-      <c r="J6" s="17"/>
-      <c r="K6" s="17"/>
-      <c r="L6" s="17"/>
-      <c r="M6" s="17"/>
-      <c r="N6" s="18"/>
+    <row r="6" customFormat="false" ht="225.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="B6" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="C6" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="D6" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="E6" s="20" t="s">
+        <v>41</v>
+      </c>
+      <c r="F6" s="17" t="s">
+        <v>42</v>
+      </c>
+      <c r="G6" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="H6" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="I6" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="J6" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="K6" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="L6" s="21" t="n">
+        <v>45984</v>
+      </c>
+      <c r="M6" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="N6" s="22" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="19"/>
-      <c r="B7" s="19"/>
-      <c r="C7" s="19"/>
-      <c r="D7" s="19"/>
-      <c r="E7" s="19"/>
-      <c r="F7" s="19"/>
-      <c r="G7" s="19"/>
-      <c r="H7" s="19"/>
-      <c r="I7" s="19"/>
-      <c r="J7" s="19"/>
-      <c r="K7" s="19"/>
-      <c r="L7" s="19"/>
-      <c r="M7" s="19"/>
-      <c r="N7" s="20"/>
+      <c r="A7" s="23"/>
+      <c r="B7" s="23"/>
+      <c r="C7" s="23"/>
+      <c r="D7" s="23"/>
+      <c r="E7" s="23"/>
+      <c r="F7" s="23"/>
+      <c r="G7" s="23"/>
+      <c r="H7" s="23"/>
+      <c r="I7" s="23"/>
+      <c r="J7" s="23"/>
+      <c r="K7" s="23"/>
+      <c r="L7" s="23"/>
+      <c r="M7" s="23"/>
+      <c r="N7" s="24"/>
     </row>
-    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="21"/>
-      <c r="B8" s="21"/>
-      <c r="C8" s="21"/>
-      <c r="D8" s="21"/>
-      <c r="E8" s="21"/>
-      <c r="F8" s="21"/>
-      <c r="G8" s="21"/>
-      <c r="H8" s="21"/>
-      <c r="I8" s="21"/>
-      <c r="J8" s="21"/>
-      <c r="K8" s="21"/>
-      <c r="L8" s="21"/>
-      <c r="M8" s="21"/>
-      <c r="N8" s="22"/>
+    <row r="8" customFormat="false" ht="166.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="25" t="s">
+        <v>47</v>
+      </c>
+      <c r="B8" s="26" t="s">
+        <v>48</v>
+      </c>
+      <c r="C8" s="25" t="s">
+        <v>49</v>
+      </c>
+      <c r="D8" s="27" t="s">
+        <v>50</v>
+      </c>
+      <c r="E8" s="27" t="s">
+        <v>51</v>
+      </c>
+      <c r="F8" s="25" t="s">
+        <v>52</v>
+      </c>
+      <c r="G8" s="25" t="s">
+        <v>53</v>
+      </c>
+      <c r="H8" s="25" t="s">
+        <v>54</v>
+      </c>
+      <c r="I8" s="25" t="s">
+        <v>21</v>
+      </c>
+      <c r="J8" s="25" t="s">
+        <v>55</v>
+      </c>
+      <c r="K8" s="25" t="s">
+        <v>34</v>
+      </c>
+      <c r="L8" s="28" t="n">
+        <v>45984</v>
+      </c>
+      <c r="M8" s="25" t="s">
+        <v>56</v>
+      </c>
+      <c r="N8" s="29"/>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="19"/>
-      <c r="B9" s="19"/>
-      <c r="C9" s="19"/>
-      <c r="D9" s="19"/>
-      <c r="E9" s="19"/>
-      <c r="F9" s="19"/>
-      <c r="G9" s="19"/>
-      <c r="H9" s="19"/>
-      <c r="I9" s="19"/>
-      <c r="J9" s="19"/>
-      <c r="K9" s="19"/>
-      <c r="L9" s="19"/>
-      <c r="M9" s="19"/>
-      <c r="N9" s="20"/>
+      <c r="A9" s="30"/>
+      <c r="B9" s="30"/>
+      <c r="C9" s="30"/>
+      <c r="D9" s="30"/>
+      <c r="E9" s="30"/>
+      <c r="F9" s="30"/>
+      <c r="G9" s="30"/>
+      <c r="H9" s="30"/>
+      <c r="I9" s="30"/>
+      <c r="J9" s="30"/>
+      <c r="K9" s="30"/>
+      <c r="L9" s="30"/>
+      <c r="M9" s="30"/>
+      <c r="N9" s="31"/>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="17"/>
@@ -894,7 +1091,7 @@
       <c r="K10" s="17"/>
       <c r="L10" s="17"/>
       <c r="M10" s="17"/>
-      <c r="N10" s="23"/>
+      <c r="N10" s="32"/>
     </row>
   </sheetData>
   <dataValidations count="2">

</xml_diff>